<commit_message>
More work on accruals
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/BIF.CO.xlsx
+++ b/data/cox_xlsx/BIF.CO.xlsx
@@ -9930,13 +9930,34 @@
       <c r="O44" s="15">
         <v>402.93</v>
       </c>
-      <c r="P44" s="16"/>
-      <c r="Q44" s="16"/>
-      <c r="R44" s="16"/>
-      <c r="S44" s="16"/>
-      <c r="T44" s="16"/>
-      <c r="U44" s="16"/>
-      <c r="V44" s="16"/>
+      <c r="P44" s="17">
+        <f t="shared" ref="P44:Q44" si="1">SUM(P46,P49,P57)</f>
+        <v>384.22</v>
+      </c>
+      <c r="Q44" s="17">
+        <f t="shared" si="1"/>
+        <v>448.15</v>
+      </c>
+      <c r="R44" s="17">
+        <f t="shared" ref="R44:T44" si="2">SUM(R46,R57)</f>
+        <v>544.11</v>
+      </c>
+      <c r="S44" s="17">
+        <f t="shared" si="2"/>
+        <v>477.01</v>
+      </c>
+      <c r="T44" s="17">
+        <f t="shared" si="2"/>
+        <v>389.05</v>
+      </c>
+      <c r="U44" s="17">
+        <f>U45</f>
+        <v>392.74</v>
+      </c>
+      <c r="V44" s="17">
+        <f>SUM(V46,V57)</f>
+        <v>389.1</v>
+      </c>
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
@@ -10656,22 +10677,27 @@
         <v>452.38</v>
       </c>
       <c r="Q62" s="19">
-        <v>467.13</v>
+        <f>467.13 + Q63</f>
+        <v>584.28</v>
       </c>
       <c r="R62" s="19">
-        <v>658.83</v>
+        <f> 658.83 + R63</f>
+        <v>738.66</v>
       </c>
       <c r="S62" s="19">
-        <v>558.68</v>
+        <f> 558.68 + S63</f>
+        <v>609.5</v>
       </c>
       <c r="T62" s="19">
-        <v>541.66</v>
+        <f> 541.66 + T63</f>
+        <v>576.96</v>
       </c>
       <c r="U62" s="19">
         <v>442.02</v>
       </c>
       <c r="V62" s="19">
-        <v>434.82</v>
+        <f> 434.82 + V63</f>
+        <v>454.07</v>
       </c>
     </row>
     <row r="63" ht="15.0" customHeight="1">

</xml_diff>